<commit_message>
v0.24: EE1(b) removed for all faculties; rename Start paper to Begin drafting
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXuBp5SMoG4pD1jWH8rtoe
</commit_message>
<xml_diff>
--- a/output/faculty_requests/ARTS - SR26 sustainability reporting request.xlsx
+++ b/output/faculty_requests/ARTS - SR26 sustainability reporting request.xlsx
@@ -686,7 +686,7 @@
     <outlinePr summaryBelow="1" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R25"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -984,46 +984,60 @@
       <c r="P16" s="15" t="n"/>
       <c r="Q16" s="15" t="n"/>
     </row>
-    <row r="17" ht="188" customHeight="1">
+    <row r="17" ht="270" customHeight="1">
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>EE1(b)</t>
+          <t>TR1(a)</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Exceptional education</t>
+          <t>Transformational research</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Provide our students with learning experiences that help them build the knowledge, skills and relationships to lead change for sustainable societies.</t>
+          <t>Utilise the expertise of the University’s researchers through mutually beneficial partnerships to help address the University’s operational sustainability challenges.</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Pilots of possible approaches for understanding and developing students’ sustainability self-efficacy</t>
+          <t>Expert-reviewed evidence of researchers contributing to operational sustainability priorities through partnerships, advisory input, living labs, applied projects or decision-support</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>Has your faculty piloted or trialled any approach in 2026 to understand or build students' confidence and capability to act on sustainability (sustainability self-efficacy)? If yes, briefly describe the approach, participating cohort, what was learned and next steps. If not, please respond 'none in 2026' – this is a new indicator and a nil response is useful.
-We are aware of the Sustainability Strengths Compass Living Lab project (CLLAP) and will collect it separately.</t>
+          <t>Please give any examples from 2026 of researchers in your faculty contributing to the University's own operational sustainability challenges (e.g. advising on campus energy, biodiversity, waste or buildings; applied projects; decision-support tools). Briefly describe the operational challenge, the researchers' contribution, the University team involved and the result.
+Please note, we will collect case studies on Campus Living Lab Accelerator Program projects directly from project owners - no need to include these.
+In end-2025 reporting your faculty reported on the related SP2030 target 2a (click the ref in Column H to see it in full in Tab 3).</t>
         </is>
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>This is a new indicator. We will use responses to establish a baseline of how (and whether) faculties are understanding student sustainability self-efficacy, and report on early pilots in the 2026 Sustainability Report. A nil response is useful to us.</t>
-        </is>
-      </c>
-      <c r="H17" s="13" t="inlineStr">
-        <is>
-          <t>N/A – new indicator</t>
-        </is>
-      </c>
-      <c r="I17" s="13" t="inlineStr"/>
-      <c r="J17" s="13" t="inlineStr"/>
-      <c r="K17" s="13" t="inlineStr"/>
+          <t>We will report on examples of researchers helping solve the University's own operational sustainability challenges, alongside Campus Living Lab Accelerator Program case studies collected directly from project owners, and share them with operational teams to identify further collaboration.</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>2a
+→ view SR25 response</t>
+        </is>
+      </c>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>Met or exceeded</t>
+        </is>
+      </c>
+      <c r="J17" s="13" t="inlineStr">
+        <is>
+          <t>See attached report. (RH note: Saved in responses folder)</t>
+        </is>
+      </c>
+      <c r="K17" s="13" t="inlineStr">
+        <is>
+          <t>Draft report on the Living Lab project is here: Report John Medley Living Lab Project FINAL.docx</t>
+        </is>
+      </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
       <c r="N17" s="15" t="n"/>
@@ -1034,7 +1048,7 @@
     <row r="18" ht="270" customHeight="1">
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>TR1(a)</t>
+          <t>TR2(a)</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
@@ -1044,29 +1058,29 @@
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Utilise the expertise of the University’s researchers through mutually beneficial partnerships to help address the University’s operational sustainability challenges.</t>
+          <t>Deliver high-quality research and partnerships that contribute to sustainability outcomes and demonstrable societal benefit.</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Expert-reviewed evidence of researchers contributing to operational sustainability priorities through partnerships, advisory input, living labs, applied projects or decision-support</t>
+          <t>Evidence of sustainability-related research impact across diverse pathways, could include policy, industry, community, practice, cultural and institutional outcomes</t>
         </is>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>Please give any examples from 2026 of researchers in your faculty contributing to the University's own operational sustainability challenges (e.g. advising on campus energy, biodiversity, waste or buildings; applied projects; decision-support tools). Briefly describe the operational challenge, the researchers' contribution, the University team involved and the result.
-Please note, we will collect case studies on Campus Living Lab Accelerator Program projects directly from project owners - no need to include these.
-In end-2025 reporting your faculty reported on the related SP2030 target 2a (click the ref in Column H to see it in full in Tab 3).</t>
+          <t>Please give any examples from 2026 of sustainability-related research from your faculty that has had impact beyond academia – on policy, industry, community, practice, cultural or institutional outcomes. Briefly describe the research, the partner or user, and the resulting change or influence, with links (e.g. Pursuit articles, policy submissions, reports).
+We will source University-wide research metrics (e.g. SDG-mapped publications via SciVal) from Melbourne Research and Enterprise (MRE) – publication counts are not required.
+In end-2025 reporting your faculty reported on the related SP2030 target 5b(i) (click the ref in Column H to see it in full in Tab 3).</t>
         </is>
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>We will report on examples of researchers helping solve the University's own operational sustainability challenges, alongside Campus Living Lab Accelerator Program case studies collected directly from project owners, and share them with operational teams to identify further collaboration.</t>
+          <t>We will collate research impact examples across faculties to show the breadth of sustainability-related research impact in the Transformational research section of the 2026 Sustainability Report, complementing University-wide metrics from Melbourne Research and Enterprise (MRE).</t>
         </is>
       </c>
       <c r="H18" s="14" t="inlineStr">
         <is>
-          <t>2a
+          <t>5b(i)
 → view SR25 response</t>
         </is>
       </c>
@@ -1077,14 +1091,10 @@
       </c>
       <c r="J18" s="13" t="inlineStr">
         <is>
-          <t>See attached report. (RH note: Saved in responses folder)</t>
-        </is>
-      </c>
-      <c r="K18" s="13" t="inlineStr">
-        <is>
-          <t>Draft report on the Living Lab project is here: Report John Medley Living Lab Project FINAL.docx</t>
-        </is>
-      </c>
+          <t>In addition to the matters listed at mid-2025, the Ass Dean joined the Board of MBI and hosted a major showcase of MBI activities to Arts Faculty researchers which boosted involvement in the BDI's researech clusters</t>
+        </is>
+      </c>
+      <c r="K18" s="13" t="inlineStr"/>
       <c r="L18" s="15" t="n"/>
       <c r="M18" s="15" t="n"/>
       <c r="N18" s="15" t="n"/>
@@ -1092,10 +1102,10 @@
       <c r="P18" s="15" t="n"/>
       <c r="Q18" s="15" t="n"/>
     </row>
-    <row r="19" ht="270" customHeight="1">
+    <row r="19" ht="237" customHeight="1">
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>TR2(a)</t>
+          <t>TR2(d)</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
@@ -1110,19 +1120,19 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Evidence of sustainability-related research impact across diverse pathways, could include policy, industry, community, practice, cultural and institutional outcomes</t>
+          <t>Case-based evidence demonstrating how research has contributed to meaningful sustainability outcomes.</t>
         </is>
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>Please give any examples from 2026 of sustainability-related research from your faculty that has had impact beyond academia – on policy, industry, community, practice, cultural or institutional outcomes. Briefly describe the research, the partner or user, and the resulting change or influence, with links (e.g. Pursuit articles, policy submissions, reports).
-We will source University-wide research metrics (e.g. SDG-mapped publications via SciVal) from Melbourne Research and Enterprise (MRE) – publication counts are not required.
+          <t>Please give any examples of research activity from your faculty that has contributed to a meaningful sustainability outcome: the research, stakeholders involved, pathway to impact and evidence of the outcome. These can be the examples from TR2(a) described in more detail.
+We are also seeking examples from Melbourne Climate Futures, the Melbourne Biodiversity Institute and Strategic Communications.
 In end-2025 reporting your faculty reported on the related SP2030 target 5b(i) (click the ref in Column H to see it in full in Tab 3).</t>
         </is>
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>We will collate research impact examples across faculties to show the breadth of sustainability-related research impact in the Transformational research section of the 2026 Sustainability Report, complementing University-wide metrics from Melbourne Research and Enterprise (MRE).</t>
+          <t>We will select the strongest examples to develop as full research case studies for the 2026 Sustainability Report (we may contact you for more detail and images).</t>
         </is>
       </c>
       <c r="H19" s="14" t="inlineStr">
@@ -1149,10 +1159,10 @@
       <c r="P19" s="15" t="n"/>
       <c r="Q19" s="15" t="n"/>
     </row>
-    <row r="20" ht="237" customHeight="1">
+    <row r="20" ht="188" customHeight="1">
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>TR2(d)</t>
+          <t>TR3(b)</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
@@ -1162,40 +1172,40 @@
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>Deliver high-quality research and partnerships that contribute to sustainability outcomes and demonstrable societal benefit.</t>
+          <t>Embed sustainability within research systems, processes, capability and culture, so research is conducted responsibly, efficiently and with reduced environmental impact.</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Case-based evidence demonstrating how research has contributed to meaningful sustainability outcomes.</t>
+          <t>Demonstrated examples of more sustainable research practices in laboratories, fieldwork, procurement, travel or infrastructure use</t>
         </is>
       </c>
       <c r="F20" s="13" t="inlineStr">
         <is>
-          <t>Please give any examples of research activity from your faculty that has contributed to a meaningful sustainability outcome: the research, stakeholders involved, pathway to impact and evidence of the outcome. These can be the examples from TR2(a) described in more detail.
-We are also seeking examples from Melbourne Climate Futures, the Melbourne Biodiversity Institute and Strategic Communications.
-In end-2025 reporting your faculty reported on the related SP2030 target 5b(i) (click the ref in Column H to see it in full in Tab 3).</t>
+          <t>Are there any efforts within the faculty to make research practices more sustainable (e.g. green lab certification, equipment sharing, reduced research travel, sustainable fieldwork, sustainable procurement of research consumables)? If so, please give any examples and any evidence of uptake, resource savings or emissions reductions.
+In end-2025 reporting your faculty reported on the related SP2030 target 5c(ii) (click the ref in Column H to see it in full in Tab 3).</t>
         </is>
       </c>
       <c r="G20" s="13" t="inlineStr">
         <is>
-          <t>We will select the strongest examples to develop as full research case studies for the 2026 Sustainability Report (we may contact you for more detail and images).</t>
+          <t>We will report on ways the University is making research practices more sustainable in the 2026 Sustainability Report, and share practical examples (e.g. green labs) across faculties.</t>
         </is>
       </c>
       <c r="H20" s="14" t="inlineStr">
         <is>
-          <t>5b(i)
+          <t>5c(ii)
 → view SR25 response</t>
         </is>
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>Met or exceeded</t>
+          <t>Not met</t>
         </is>
       </c>
       <c r="J20" s="13" t="inlineStr">
         <is>
-          <t>In addition to the matters listed at mid-2025, the Ass Dean joined the Board of MBI and hosted a major showcase of MBI activities to Arts Faculty researchers which boosted involvement in the BDI's researech clusters</t>
+          <t>This needs more specific attention
+In general terms, the Faculty has focused on reducing air travel, the major environmental impact of our research activity.</t>
         </is>
       </c>
       <c r="K20" s="13" t="inlineStr"/>
@@ -1209,50 +1219,50 @@
     <row r="21" ht="188" customHeight="1">
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>TR3(b)</t>
+          <t>EN1(a)</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>Transformational research</t>
+          <t>Enablers</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Embed sustainability within research systems, processes, capability and culture, so research is conducted responsibly, efficiently and with reduced environmental impact.</t>
+          <t>Enablers</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Demonstrated examples of more sustainable research practices in laboratories, fieldwork, procurement, travel or infrastructure use</t>
+          <t>Evidence of sustainability outcomes informed by Indigenous knowledges</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>Are there any efforts within the faculty to make research practices more sustainable (e.g. green lab certification, equipment sharing, reduced research travel, sustainable fieldwork, sustainable procurement of research consumables)? If so, please give any examples and any evidence of uptake, resource savings or emissions reductions.
-In end-2025 reporting your faculty reported on the related SP2030 target 5c(ii) (click the ref in Column H to see it in full in Tab 3).</t>
+          <t>Please give any examples of activity in your faculty (education, research, engagement or operations) where Indigenous knowledges informed a sustainability outcome. Describe the activity, how Indigenous knowledges were incorporated or co-created and with whom, and the result. Please confirm that appropriate permissions are in place for sharing.
+In end-2025 reporting your faculty reported on the related SP2030 target 6a (click the ref in Column H to see it in full in Tab 3).</t>
         </is>
       </c>
       <c r="G21" s="13" t="inlineStr">
         <is>
-          <t>We will report on ways the University is making research practices more sustainable in the 2026 Sustainability Report, and share practical examples (e.g. green labs) across faculties.</t>
+          <t>We will report on the ways Indigenous knowledges inform sustainability activities across the University, and develop selected examples into case studies with appropriate permissions.</t>
         </is>
       </c>
       <c r="H21" s="14" t="inlineStr">
         <is>
-          <t>5c(ii)
+          <t>6a
 → view SR25 response</t>
         </is>
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
-          <t>Not met</t>
+          <t>Partially met</t>
         </is>
       </c>
       <c r="J21" s="13" t="inlineStr">
         <is>
-          <t>This needs more specific attention
-In general terms, the Faculty has focused on reducing air travel, the major environmental impact of our research activity.</t>
+          <t>See previous response. (copied below) 
+In addition to housing the Indigenous Studies Program, academic staff have contributed to University-wide Indigenous-led initiatives with important sustainability consequences, and more broadly, champsion such values in their scholarly work.</t>
         </is>
       </c>
       <c r="K21" s="13" t="inlineStr"/>
@@ -1263,10 +1273,10 @@
       <c r="P21" s="15" t="n"/>
       <c r="Q21" s="15" t="n"/>
     </row>
-    <row r="22" ht="188" customHeight="1">
+    <row r="22" ht="220" customHeight="1">
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>EN1(a)</t>
+          <t>EN1(b)</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
@@ -1281,38 +1291,42 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Evidence of sustainability outcomes informed by Indigenous knowledges</t>
+          <t>Living laboratories enabling applied learning, research and operational sustainability outcomes</t>
         </is>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
-          <t>Please give any examples of activity in your faculty (education, research, engagement or operations) where Indigenous knowledges informed a sustainability outcome. Describe the activity, how Indigenous knowledges were incorporated or co-created and with whom, and the result. Please confirm that appropriate permissions are in place for sharing.
-In end-2025 reporting your faculty reported on the related SP2030 target 6a (click the ref in Column H to see it in full in Tab 3).</t>
+          <t>Please give any examples of sustainability-related living labs operating within your faculty in 2026 – their activities, who is involved (students, researchers, operational staff) and their outputs, outcomes or impact.
+Please note, we will collect case studies on Campus Living Lab Accelerator Program projects directly from project owners - no need to include these.
+In end-2025 reporting your faculty reported on the related SP2030 target 2a (click the ref in Column H to see it in full in Tab 3).</t>
         </is>
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>We will report on the ways Indigenous knowledges inform sustainability activities across the University, and develop selected examples into case studies with appropriate permissions.</t>
+          <t>We will share examples of sustainability-related living labs from across the University in the 2026 Sustainability Report, alongside Campus Living Lab Accelerator Program case studies collected directly from project owners.</t>
         </is>
       </c>
       <c r="H22" s="14" t="inlineStr">
         <is>
-          <t>6a
+          <t>2a
 → view SR25 response</t>
         </is>
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>Partially met</t>
+          <t>Met or exceeded</t>
         </is>
       </c>
       <c r="J22" s="13" t="inlineStr">
         <is>
-          <t>See previous response. (copied below) 
-In addition to housing the Indigenous Studies Program, academic staff have contributed to University-wide Indigenous-led initiatives with important sustainability consequences, and more broadly, champsion such values in their scholarly work.</t>
-        </is>
-      </c>
-      <c r="K22" s="13" t="inlineStr"/>
+          <t>See attached report. (RH note: Saved in responses folder)</t>
+        </is>
+      </c>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>Draft report on the Living Lab project is here: Report John Medley Living Lab Project FINAL.docx</t>
+        </is>
+      </c>
       <c r="L22" s="15" t="n"/>
       <c r="M22" s="15" t="n"/>
       <c r="N22" s="15" t="n"/>
@@ -1320,10 +1334,10 @@
       <c r="P22" s="15" t="n"/>
       <c r="Q22" s="15" t="n"/>
     </row>
-    <row r="23" ht="220" customHeight="1">
+    <row r="23" ht="154" customHeight="1">
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>EN1(b)</t>
+          <t>EN1(c)</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
@@ -1338,42 +1352,37 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Living laboratories enabling applied learning, research and operational sustainability outcomes</t>
+          <t>Coordinated internal engagement and external partnerships contributing to delivery of sustainability outcomes across priority areas.</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>Please give any examples of sustainability-related living labs operating within your faculty in 2026 – their activities, who is involved (students, researchers, operational staff) and their outputs, outcomes or impact.
-Please note, we will collect case studies on Campus Living Lab Accelerator Program projects directly from project owners - no need to include these.
-In end-2025 reporting your faculty reported on the related SP2030 target 2a (click the ref in Column H to see it in full in Tab 3).</t>
+          <t>Please list the key sustainability-focused communities of practice, internal networks or external partnerships active in your faculty in 2026 (name, partners, priority area), and give any examples of activity that contributed to a Sustainability 2030 outcome.
+In end-2025 reporting your faculty reported on the related SP2030 target 3a(ii) (click the ref in Column H to see it in full in Tab 3).</t>
         </is>
       </c>
       <c r="G23" s="13" t="inlineStr">
         <is>
-          <t>We will share examples of sustainability-related living labs from across the University in the 2026 Sustainability Report, alongside Campus Living Lab Accelerator Program case studies collected directly from project owners.</t>
+          <t>We will report on internal engagement and partnerships contributing to Sustainability 2030 outcomes, and update our record of sustainability-focused communities of practice and contacts across the University.</t>
         </is>
       </c>
       <c r="H23" s="14" t="inlineStr">
         <is>
-          <t>2a
+          <t>3a(ii)
 → view SR25 response</t>
         </is>
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>Met or exceeded</t>
+          <t>Partially met</t>
         </is>
       </c>
       <c r="J23" s="13" t="inlineStr">
         <is>
-          <t>See attached report. (RH note: Saved in responses folder)</t>
-        </is>
-      </c>
-      <c r="K23" s="13" t="inlineStr">
-        <is>
-          <t>Draft report on the Living Lab project is here: Report John Medley Living Lab Project FINAL.docx</t>
-        </is>
-      </c>
+          <t>Academics in the Faculty have supported and learned from each other in new ways through the Living Lab and through using the sustainability networks in the Faculty and beyond to showcase and develop T&amp;L initiatives. This is, of course, an ongoing process.</t>
+        </is>
+      </c>
+      <c r="K23" s="13" t="inlineStr"/>
       <c r="L23" s="15" t="n"/>
       <c r="M23" s="15" t="n"/>
       <c r="N23" s="15" t="n"/>
@@ -1381,63 +1390,7 @@
       <c r="P23" s="15" t="n"/>
       <c r="Q23" s="15" t="n"/>
     </row>
-    <row r="24" ht="154" customHeight="1">
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>EN1(c)</t>
-        </is>
-      </c>
-      <c r="C24" s="12" t="inlineStr">
-        <is>
-          <t>Enablers</t>
-        </is>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
-        <is>
-          <t>Enablers</t>
-        </is>
-      </c>
-      <c r="E24" s="12" t="inlineStr">
-        <is>
-          <t>Coordinated internal engagement and external partnerships contributing to delivery of sustainability outcomes across priority areas.</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
-        <is>
-          <t>Please list the key sustainability-focused communities of practice, internal networks or external partnerships active in your faculty in 2026 (name, partners, priority area), and give any examples of activity that contributed to a Sustainability 2030 outcome.
-In end-2025 reporting your faculty reported on the related SP2030 target 3a(ii) (click the ref in Column H to see it in full in Tab 3).</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="inlineStr">
-        <is>
-          <t>We will report on internal engagement and partnerships contributing to Sustainability 2030 outcomes, and update our record of sustainability-focused communities of practice and contacts across the University.</t>
-        </is>
-      </c>
-      <c r="H24" s="14" t="inlineStr">
-        <is>
-          <t>3a(ii)
-→ view SR25 response</t>
-        </is>
-      </c>
-      <c r="I24" s="13" t="inlineStr">
-        <is>
-          <t>Partially met</t>
-        </is>
-      </c>
-      <c r="J24" s="13" t="inlineStr">
-        <is>
-          <t>Academics in the Faculty have supported and learned from each other in new ways through the Living Lab and through using the sustainability networks in the Faculty and beyond to showcase and develop T&amp;L initiatives. This is, of course, an ongoing process.</t>
-        </is>
-      </c>
-      <c r="K24" s="13" t="inlineStr"/>
-      <c r="L24" s="15" t="n"/>
-      <c r="M24" s="15" t="n"/>
-      <c r="N24" s="15" t="n"/>
-      <c r="O24" s="15" t="n"/>
-      <c r="P24" s="15" t="n"/>
-      <c r="Q24" s="15" t="n"/>
-    </row>
-    <row r="25"/>
+    <row r="24"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <mergeCells count="4">
@@ -1447,19 +1400,19 @@
     <mergeCell ref="B4:C8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="P16:P24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Please select from the dropdown" type="list">
+    <dataValidation sqref="P16:P23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Please select from the dropdown" type="list">
       <formula1>=Lists!$C$2:$C$4</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="H16" location="'3. SR25 responses'!B12"/>
-    <hyperlink ref="H18" location="'3. SR25 responses'!B8"/>
+    <hyperlink ref="H17" location="'3. SR25 responses'!B8"/>
+    <hyperlink ref="H18" location="'3. SR25 responses'!B14"/>
     <hyperlink ref="H19" location="'3. SR25 responses'!B14"/>
-    <hyperlink ref="H20" location="'3. SR25 responses'!B14"/>
-    <hyperlink ref="H21" location="'3. SR25 responses'!B15"/>
-    <hyperlink ref="H22" location="'3. SR25 responses'!B16"/>
-    <hyperlink ref="H23" location="'3. SR25 responses'!B8"/>
-    <hyperlink ref="H24" location="'3. SR25 responses'!B10"/>
+    <hyperlink ref="H20" location="'3. SR25 responses'!B15"/>
+    <hyperlink ref="H21" location="'3. SR25 responses'!B16"/>
+    <hyperlink ref="H22" location="'3. SR25 responses'!B8"/>
+    <hyperlink ref="H23" location="'3. SR25 responses'!B10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>